<commit_message>
chore: update schedule data to week of 2026-05-11 and refresh output reports
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -525,7 +525,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Max Score  |  Week of 2026-05-04</t>
+          <t>Copper &amp; Cloves  |  Max Score  |  Week of 2026-05-11</t>
         </is>
       </c>
     </row>
@@ -538,43 +538,43 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-4-May</t>
+11-May</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-5-May</t>
+12-May</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-6-May</t>
+13-May</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-7-May</t>
+14-May</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-8-May</t>
+15-May</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-9-May</t>
+16-May</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-10-May</t>
+17-May</t>
         </is>
       </c>
     </row>
@@ -626,7 +626,14 @@
           <t>09:30</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+10% pred | 10% hist
+[CONSIDER]</t>
+        </is>
+      </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
@@ -738,19 +745,12 @@
           <t>20:00</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
+      <c r="B10" s="5" t="n"/>
       <c r="C10" s="5" t="n"/>
       <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
-Kajol Kanchan
+Shruti Kulkarni
 20% pred | 0% hist
 [EXPERIMENTAL]</t>
         </is>
@@ -790,7 +790,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Trainer Hours  |  Week of 2026-05-04</t>
+          <t>Copper &amp; Cloves  |  Trainer Hours  |  Week of 2026-05-11</t>
         </is>
       </c>
     </row>
@@ -803,57 +803,78 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-4-May</t>
+11-May</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-5-May</t>
+12-May</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-6-May</t>
+13-May</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-7-May</t>
+14-May</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-8-May</t>
+15-May</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-9-May</t>
+16-May</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-10-May</t>
+17-May</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
-      <c r="A3" s="7" t="inlineStr">
-        <is>
-          <t>09:00</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
         </is>
       </c>
       <c r="B3" s="5" t="n"/>
       <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Chaitanya Nahar
+18% pred | 18% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
       <c r="E3" s="5" t="n"/>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+      <c r="H3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="5" t="n"/>
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
@@ -861,56 +882,28 @@
 [EXPERIMENTAL]</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
     </row>
     <row r="5" ht="52" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
       <c r="F5" s="5" t="n"/>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
@@ -922,14 +915,7 @@
       <c r="B6" s="5" t="n"/>
       <c r="C6" s="5" t="n"/>
       <c r="D6" s="5" t="n"/>
-      <c r="E6" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
+      <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="6" t="inlineStr">
         <is>
@@ -939,7 +925,14 @@
 [CONSIDER]</t>
         </is>
       </c>
-      <c r="H6" s="5" t="n"/>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Siddhartha Kusuma
+20% pred | 20% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -1046,7 +1039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1062,7 +1055,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Class Variety  |  Week of 2026-05-04</t>
+          <t>Copper &amp; Cloves  |  Class Variety  |  Week of 2026-05-11</t>
         </is>
       </c>
     </row>
@@ -1075,43 +1068,43 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-4-May</t>
+11-May</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-5-May</t>
+12-May</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-6-May</t>
+13-May</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-7-May</t>
+14-May</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-8-May</t>
+15-May</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-9-May</t>
+16-May</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-10-May</t>
+17-May</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1174,7 @@
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -1189,20 +1182,27 @@
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+100% pred | 100% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="n"/>
+Siddhartha Kusuma
+20% pred | 20% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B7" s="5" t="n"/>
@@ -1210,75 +1210,47 @@
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-100% pred | 100% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n"/>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>18:15</t>
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+17% pred | 17% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
     </row>
     <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
-        <is>
-          <t>18:15</t>
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="5" t="n"/>
       <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="E9" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
@@ -1286,37 +1258,37 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
+      <c r="F9" s="5" t="n"/>
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="52" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
feat: add diagnostic test scripts for schedule data and implement UI enhancements including a global loader and improved grid stickiness.
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -626,14 +626,7 @@
           <t>09:30</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-10% pred | 10% hist
-[CONSIDER]</t>
-        </is>
-      </c>
+      <c r="B5" s="5" t="n"/>
       <c r="C5" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
@@ -745,7 +738,14 @@
           <t>20:00</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
       <c r="C10" s="5" t="n"/>
       <c r="D10" s="8" t="inlineStr">
         <is>
@@ -774,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -909,7 +909,7 @@
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
@@ -917,27 +917,20 @@
       <c r="D6" s="5" t="n"/>
       <c r="E6" s="5" t="n"/>
       <c r="F6" s="5" t="n"/>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-100% pred | 100% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
+      <c r="G6" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+Shruti Kulkarni
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>18:00</t>
+          <t>11:30</t>
         </is>
       </c>
       <c r="B7" s="5" t="n"/>
@@ -945,27 +938,55 @@
       <c r="D7" s="5" t="n"/>
       <c r="E7" s="5" t="n"/>
       <c r="F7" s="5" t="n"/>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="n"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+100% pred | 100% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Siddhartha Kusuma
+20% pred | 20% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>18:00</t>
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="5" t="n"/>
       <c r="D8" s="5" t="n"/>
       <c r="E8" s="5" t="n"/>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="5" t="n"/>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="5" t="n"/>
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
@@ -973,19 +994,19 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="5" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
@@ -993,37 +1014,37 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
       <c r="H10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>20:00</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n"/>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Shruti Kulkarni
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="5" t="n"/>
+      <c r="H11" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
refactor: update scheduling data and optimization logic for the week of May 4th to 10th
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -47,13 +47,13 @@
       <sz val="9"/>
     </font>
     <font>
+      <color rgb="006B21A8"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <b val="1"/>
       <color rgb="0092400E"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="006B21A8"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="8">
@@ -75,22 +75,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00D5F2F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FAFAFA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D5F2F8"/>
+        <fgColor rgb="00E8D5FF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFBEB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8D5FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,15 +134,15 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -525,7 +525,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Max Score  |  Week of 2026-05-11</t>
+          <t>Copper &amp; Cloves  |  Max Score  |  Week of 2026-05-04</t>
         </is>
       </c>
     </row>
@@ -538,227 +538,283 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-11-May</t>
+4-May</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-12-May</t>
+5-May</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-13-May</t>
+6-May</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-14-May</t>
+7-May</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-15-May</t>
+8-May</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-16-May</t>
+9-May</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-17-May</t>
+10-May</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:15</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Chaitanya Nahar
-18% pred | 18% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+12% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Pushyank Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
-100% pred | 100% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
 Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="8" t="inlineStr">
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Kajol Kanchan
+10% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Siddhartha Kusuma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Chaitanya Nahar
+100% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
 20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="n"/>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+[]</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+28% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -790,7 +846,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Trainer Hours  |  Week of 2026-05-11</t>
+          <t>Copper &amp; Cloves  |  Trainer Hours  |  Week of 2026-05-04</t>
         </is>
       </c>
     </row>
@@ -803,248 +859,283 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-11-May</t>
+4-May</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-12-May</t>
+5-May</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-13-May</t>
+6-May</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-14-May</t>
+7-May</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-15-May</t>
+8-May</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-16-May</t>
+9-May</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-17-May</t>
+10-May</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:15</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Chaitanya Nahar
-18% pred | 18% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+12% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Pushyank Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>10:15</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="n"/>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-100% pred | 100% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
 Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Kajol Kanchan
+10% pred | 0% hist
+[]</t>
         </is>
       </c>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="8" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Siddhartha Kusuma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Chaitanya Nahar
+100% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
 20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="7" t="inlineStr">
+[]</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+28% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="8" t="inlineStr">
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-    </row>
-    <row r="11" ht="52" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="n"/>
-      <c r="D11" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="n"/>
-      <c r="G11" s="5" t="n"/>
-      <c r="H11" s="5" t="n"/>
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1060,7 +1151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1076,7 +1167,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Class Variety  |  Week of 2026-05-11</t>
+          <t>Copper &amp; Cloves  |  Class Variety  |  Week of 2026-05-04</t>
         </is>
       </c>
     </row>
@@ -1089,227 +1180,283 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-11-May</t>
+4-May</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-12-May</t>
+5-May</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-13-May</t>
+6-May</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-14-May</t>
+7-May</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-15-May</t>
+8-May</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-16-May</t>
+9-May</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-17-May</t>
+10-May</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>08:15</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Chaitanya Nahar
-18% pred | 18% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="5" t="n"/>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+12% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Pushyank Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Siddhartha Kusuma
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Pushyank Nahar
-100% pred | 100% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="H6" s="8" t="inlineStr">
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
 Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="8" t="inlineStr">
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Kajol Kanchan
+10% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Siddhartha Kusuma
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Chaitanya Nahar
+100% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
 20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H7" s="5" t="n"/>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+[]</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+28% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>20:00</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+15% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
refactor: enhance availability settings UI and improve responsiveness
- Adjusted availability grid layout for better responsiveness and usability.
- Updated table styles for improved readability and consistency.
- Simplified time input fields and adjusted padding for a cleaner look.
- Added location abbreviation mapping for better display of studio names.
- Improved interaction feedback for availability toggles
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -39,7 +39,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00555577"/>
+      <color rgb="0092400E"/>
       <sz val="10"/>
     </font>
     <font>
@@ -47,13 +47,13 @@
       <sz val="9"/>
     </font>
     <font>
-      <b val="1"/>
-      <color rgb="0092400E"/>
-      <sz val="10"/>
+      <color rgb="000C4A6E"/>
+      <sz val="9"/>
     </font>
     <font>
-      <color rgb="000C4A6E"/>
-      <sz val="9"/>
+      <b val="1"/>
+      <color rgb="00555577"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="8">
@@ -70,7 +70,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F8"/>
+        <fgColor rgb="00FFFBEB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8D5FF"/>
       </patternFill>
     </fill>
     <fill>
@@ -80,17 +85,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8D5FF"/>
+        <fgColor rgb="00D5F2F8"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFBEB"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D5F2F8"/>
+        <fgColor rgb="00F5F5F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -134,15 +134,15 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -525,7 +525,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Max Score  |  Week of 2026-05-11</t>
+          <t>Copper &amp; Cloves  |  Max Score  |  Week of 2026-05-04</t>
         </is>
       </c>
     </row>
@@ -538,147 +538,64 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-11-May</t>
+4-May</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-12-May</t>
+5-May</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-13-May</t>
+6-May</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-14-May</t>
+7-May</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-15-May</t>
+8-May</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-16-May</t>
+9-May</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-17-May</t>
+10-May</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>07:30</t>
-        </is>
-      </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
 Chaitanya Nahar
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>09:00</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Pushyank Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>10:15</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="n"/>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="6" t="inlineStr">
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
 Siddhartha Kusuma
@@ -686,8 +603,7 @@
 [EXPERIMENTAL]</t>
         </is>
       </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="8" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Siddhartha Kusuma
@@ -695,46 +611,67 @@
 [CONSIDER]</t>
         </is>
       </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>18:00</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
+85% pred | 85% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Siddhartha Kusuma
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="6" t="n"/>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
 Chaitanya Nahar
 20% pred | 0% hist
 [EXPERIMENTAL]</t>
         </is>
       </c>
-      <c r="H8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="5" t="n"/>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
@@ -742,37 +679,51 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="F9" s="5" t="n"/>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
-    </row>
-    <row r="10" ht="52" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Chaitanya Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Chaitanya Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -788,7 +739,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -804,7 +755,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Trainer Hours  |  Week of 2026-05-11</t>
+          <t>Copper &amp; Cloves  |  Trainer Hours  |  Week of 2026-05-04</t>
         </is>
       </c>
     </row>
@@ -817,57 +768,57 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-11-May</t>
+4-May</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-12-May</t>
+5-May</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-13-May</t>
+6-May</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-14-May</t>
+7-May</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-15-May</t>
+8-May</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-16-May</t>
+9-May</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-17-May</t>
+10-May</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
@@ -875,75 +826,27 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
 Chaitanya Nahar
 20% pred | 0% hist
 [EXPERIMENTAL]</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-24% pred | 24% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>10:15</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
 Siddhartha Kusuma
@@ -951,8 +854,7 @@
 [EXPERIMENTAL]</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Siddhartha Kusuma
@@ -960,46 +862,67 @@
 [CONSIDER]</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+85% pred | 85% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Siddhartha Kusuma
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Chaitanya Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
@@ -1007,44 +930,30 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Kajol Kanchan
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Kajol Kanchan
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Chaitanya Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1060,7 +969,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1076,7 +985,7 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Copper &amp; Cloves  |  Class Variety  |  Week of 2026-05-11</t>
+          <t>Copper &amp; Cloves  |  Class Variety  |  Week of 2026-05-04</t>
         </is>
       </c>
     </row>
@@ -1089,57 +998,57 @@
       <c r="B2" s="3" t="inlineStr">
         <is>
           <t>Monday
-11-May</t>
+4-May</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Tuesday
-12-May</t>
+5-May</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
           <t>Wednesday
-13-May</t>
+6-May</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Thursday
-14-May</t>
+7-May</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Friday
-15-May</t>
+8-May</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Saturday
-16-May</t>
+9-May</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Sunday
-17-May</t>
+10-May</t>
         </is>
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="8" t="inlineStr">
         <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
@@ -1147,75 +1056,27 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
-        <is>
-          <t>09:30</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
 Chaitanya Nahar
 20% pred | 0% hist
 [EXPERIMENTAL]</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-24% pred | 24% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>10:15</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Shruti Kulkarni
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="7" t="inlineStr">
-        <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
 Siddhartha Kusuma
@@ -1223,8 +1084,7 @@
 [EXPERIMENTAL]</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="8" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Siddhartha Kusuma
@@ -1232,46 +1092,67 @@
 [CONSIDER]</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="5" t="n"/>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
-    </row>
-    <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+85% pred | 85% hist
+[CONSIDER]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Siddhartha Kusuma
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="6" t="n"/>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Chaitanya Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
@@ -1279,44 +1160,30 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="52" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n"/>
-      <c r="D9" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Kajol Kanchan
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="n"/>
-      <c r="F9" s="8" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Mat 57
-Kajol Kanchan
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="G9" s="5" t="n"/>
-      <c r="H9" s="5" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Chaitanya Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Apply scheduler rules and settings persistence updates
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -39,20 +39,20 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="0092400E"/>
+      <color rgb="00555577"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="000C4A6E"/>
+      <sz val="9"/>
     </font>
     <font>
       <color rgb="006B21A8"/>
       <sz val="9"/>
     </font>
     <font>
-      <color rgb="000C4A6E"/>
-      <sz val="9"/>
-    </font>
-    <font>
       <b val="1"/>
-      <color rgb="00555577"/>
+      <color rgb="0092400E"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -70,7 +70,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFBEB"/>
+        <fgColor rgb="00F5F5F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F2F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FAFAFA"/>
       </patternFill>
     </fill>
     <fill>
@@ -80,17 +90,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FAFAFA"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D5F2F8"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F5F5F8"/>
+        <fgColor rgb="00FFFBEB"/>
       </patternFill>
     </fill>
   </fills>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -581,112 +581,98 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>07:00</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>Copper + Cloves FIT
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+12% pred | 0% hist
+[]</t>
         </is>
       </c>
       <c r="C3" s="6" t="n"/>
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="n"/>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Siddhartha Kusuma
-100% pred | 100% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="H3" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-85% pred | 85% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
       <c r="G5" s="6" t="n"/>
-      <c r="H5" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
+      <c r="H5" s="6" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
-      <c r="E6" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
 Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="n"/>
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G6" s="6" t="n"/>
       <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>20:00</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
@@ -694,36 +680,113 @@
       <c r="D7" s="6" t="n"/>
       <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
-      <c r="G7" s="5" t="inlineStr">
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="n"/>
+Siddhartha Kusuma
+10% pred | 0% hist
+[]</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>20:15</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>11:15</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
-      <c r="F8" s="7" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Pushyank Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="n"/>
-      <c r="H8" s="6" t="n"/>
+100% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -739,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -809,151 +872,214 @@
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>07:30</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="n"/>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+12% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C3" s="6" t="n"/>
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="n"/>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+      <c r="F3" s="6" t="n"/>
       <c r="G3" s="6" t="n"/>
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
       <c r="C4" s="6" t="n"/>
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Siddhartha Kusuma
-100% pred | 100% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-85% pred | 85% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n"/>
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G6" s="6" t="n"/>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
+      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+      <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Siddhartha Kusuma
+10% pred | 0% hist
+[]</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>20:00</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>11:15</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Pushyank Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F8" s="6" t="n"/>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
 Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="n"/>
+100% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -969,7 +1095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1039,151 +1165,214 @@
       </c>
     </row>
     <row r="3" ht="52" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t>07:30</t>
-        </is>
-      </c>
-      <c r="B3" s="6" t="n"/>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+12% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C3" s="6" t="n"/>
       <c r="D3" s="6" t="n"/>
       <c r="E3" s="6" t="n"/>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-17% pred | 17% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+      <c r="F3" s="6" t="n"/>
       <c r="G3" s="6" t="n"/>
       <c r="H3" s="6" t="n"/>
     </row>
     <row r="4" ht="52" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>11:30</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
+          <t>07:30</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n"/>
       <c r="C4" s="6" t="n"/>
       <c r="D4" s="6" t="n"/>
       <c r="E4" s="6" t="n"/>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Copper + Cloves Mat 57
 Siddhartha Kusuma
-100% pred | 100% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Siddhartha Kusuma
-85% pred | 85% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t>12:00</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Siddhartha Kusuma
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="n"/>
+18% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
       <c r="G5" s="6" t="n"/>
       <c r="H5" s="6" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
-        <is>
-          <t>18:15</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="n"/>
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="C6" s="6" t="n"/>
       <c r="D6" s="6" t="n"/>
       <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="G6" s="6" t="n"/>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves FIT
-Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
+      <c r="H6" s="6" t="n"/>
     </row>
     <row r="7" ht="52" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="B7" s="6" t="n"/>
       <c r="C7" s="6" t="n"/>
       <c r="D7" s="6" t="n"/>
-      <c r="E7" s="5" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
+      <c r="E7" s="6" t="n"/>
       <c r="F7" s="6" t="n"/>
       <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Siddhartha Kusuma
+10% pred | 0% hist
+[]</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="52" customHeight="1">
-      <c r="A8" s="8" t="inlineStr">
-        <is>
-          <t>20:00</t>
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>11:15</t>
         </is>
       </c>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="6" t="n"/>
-      <c r="E8" s="6" t="n"/>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves FIT
+Pushyank Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
       <c r="F8" s="6" t="n"/>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
+Kajol Kanchan
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
 Chaitanya Nahar
-20% pred | 0% hist
-[EXPERIMENTAL]</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="n"/>
+100% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+20% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="52" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+17% pred | 0% hist
+[]</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Refine planner UI and schedule controls
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -609,67 +609,46 @@
       </c>
     </row>
     <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>17:00</t>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>18:15</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-8% pred | 8% hist
-[CONSIDER]</t>
-        </is>
-      </c>
+Siddhartha Kusuma
+17% pred | 17% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
+Kajol Kanchan
+15% pred | 15% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n"/>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -685,7 +664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -820,44 +799,23 @@
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
+Kajol Kanchan
+15% pred | 15% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n"/>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -873,7 +831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -985,67 +943,46 @@
       </c>
     </row>
     <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>17:00</t>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>18:15</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
       <c r="C5" s="5" t="n"/>
       <c r="D5" s="5" t="n"/>
       <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-8% pred | 8% hist
-[CONSIDER]</t>
-        </is>
-      </c>
+Siddhartha Kusuma
+17% pred | 17% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n"/>
       <c r="H5" s="5" t="n"/>
     </row>
     <row r="6" ht="52" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>19:45</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
-Chaitanya Nahar
-20% pred | 20% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="5" t="n"/>
+Kajol Kanchan
+15% pred | 15% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
       <c r="H6" s="5" t="n"/>
-    </row>
-    <row r="7" ht="52" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>19:45</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="n"/>
-      <c r="C7" s="5" t="n"/>
-      <c r="D7" s="5" t="n"/>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Copper + Cloves Barre 57
-Kajol Kanchan
-15% pred | 15% hist
-[PROTECT_EXACT]</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n"/>
-      <c r="G7" s="5" t="n"/>
-      <c r="H7" s="5" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Improve derived studio scheduling
</commit_message>
<xml_diff>
--- a/outputs/schedule_copper_cloves.xlsx
+++ b/outputs/schedule_copper_cloves.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,10 @@
       <sz val="10"/>
     </font>
     <font>
+      <color rgb="000C4A6E"/>
+      <sz val="9"/>
+    </font>
+    <font>
       <color rgb="006B21A8"/>
       <sz val="9"/>
     </font>
@@ -52,7 +56,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +71,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F5F5F8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D5F2F8"/>
       </patternFill>
     </fill>
     <fill>
@@ -111,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -125,11 +134,14 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -497,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -569,14 +581,35 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+12% pred | 12% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
@@ -584,22 +617,71 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 46% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Pushyank Nahar
+21% pred | 21% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>11:30</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
 Siddhartha Kusuma
@@ -608,17 +690,45 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+20% pred | 20% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+28% pred | 28% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
@@ -626,19 +736,19 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
@@ -646,9 +756,9 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -664,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -736,14 +846,35 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+12% pred | 12% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
@@ -751,22 +882,71 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 46% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Pushyank Nahar
+21% pred | 21% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>11:30</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
 Siddhartha Kusuma
@@ -775,37 +955,65 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="5" t="n"/>
-      <c r="G5" s="6" t="inlineStr">
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
-8% pred | 8% hist
-[CONSIDER]</t>
-        </is>
-      </c>
-      <c r="H5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+20% pred | 20% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+28% pred | 28% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Siddhartha Kusuma
+17% pred | 17% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
@@ -813,9 +1021,9 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -831,7 +1039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -903,14 +1111,35 @@
     <row r="3" ht="52" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
+          <t>07:00</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+12% pred | 12% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="n"/>
+      <c r="D3" s="6" t="n"/>
+      <c r="E3" s="6" t="n"/>
+      <c r="F3" s="6" t="n"/>
+      <c r="G3" s="6" t="n"/>
+      <c r="H3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="52" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
           <t>07:30</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n"/>
-      <c r="C3" s="5" t="n"/>
-      <c r="D3" s="5" t="n"/>
-      <c r="E3" s="5" t="n"/>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="B4" s="6" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="6" t="n"/>
+      <c r="E4" s="6" t="n"/>
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Chaitanya Nahar
@@ -918,22 +1147,71 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="G3" s="5" t="n"/>
-      <c r="H3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="52" customHeight="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="G4" s="6" t="n"/>
+      <c r="H4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="52" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+20% pred | 0% hist
+[EXPERIMENTAL]</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+      <c r="F5" s="6" t="n"/>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Pushyank Nahar
+46% pred | 46% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="52" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Pushyank Nahar
+21% pred | 21% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+      <c r="H6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="52" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>11:30</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n"/>
-      <c r="C4" s="5" t="n"/>
-      <c r="D4" s="5" t="n"/>
-      <c r="E4" s="5" t="n"/>
-      <c r="F4" s="5" t="n"/>
-      <c r="G4" s="5" t="n"/>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+      <c r="F7" s="6" t="n"/>
+      <c r="G7" s="6" t="n"/>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves FIT
 Siddhartha Kusuma
@@ -942,17 +1220,45 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="52" customHeight="1">
-      <c r="A5" s="7" t="inlineStr">
+    <row r="8" ht="52" customHeight="1">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Barre 57
+Chaitanya Nahar
+20% pred | 20% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>Copper + Cloves Mat 57
+Shruti Kulkarni
+28% pred | 28% hist
+[PROTECT_EXACT]</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="52" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>18:15</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n"/>
-      <c r="C5" s="5" t="n"/>
-      <c r="D5" s="5" t="n"/>
-      <c r="E5" s="5" t="n"/>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Siddhartha Kusuma
@@ -960,19 +1266,19 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="G5" s="5" t="n"/>
-      <c r="H5" s="5" t="n"/>
-    </row>
-    <row r="6" ht="52" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="52" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n"/>
-      <c r="C6" s="5" t="n"/>
-      <c r="D6" s="5" t="n"/>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>Copper + Cloves Barre 57
 Kajol Kanchan
@@ -980,9 +1286,9 @@
 [PROTECT_EXACT]</t>
         </is>
       </c>
-      <c r="F6" s="5" t="n"/>
-      <c r="G6" s="5" t="n"/>
-      <c r="H6" s="5" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>